<commit_message>
feat: Configure SharePoint ID discovery script with actual Microsoft Entra ID credentials, capture execution logs, and extract SharePoint data.
</commit_message>
<xml_diff>
--- a/dados_sharepoint/colaboradores_inativos.xlsx
+++ b/dados_sharepoint/colaboradores_inativos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos IA\Kotrik\mcs-personal\dados_sharepoint\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E1CFCF6-5CAD-4D02-B8D9-3EDA572EFAFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23CA95FC-A1C4-41C0-A0D0-59F4ED4CCDA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1DDAD55E-97D1-4860-9ADC-7095B84C1F33}"/>
   </bookViews>
@@ -1437,7 +1437,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.109375" customWidth="1"/>
-    <col min="2" max="2" width="13.21875" customWidth="1"/>
+    <col min="2" max="2" width="27" customWidth="1"/>
     <col min="6" max="6" width="11.33203125" customWidth="1"/>
     <col min="7" max="7" width="13.109375" customWidth="1"/>
     <col min="8" max="8" width="9.44140625" customWidth="1"/>

</xml_diff>